<commit_message>
udpated week 3 first lecture
</commit_message>
<xml_diff>
--- a/Week02/02-Finance_and_logical functions.xlsx
+++ b/Week02/02-Finance_and_logical functions.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Dhruv\Downloads\BA-L\Week02\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{3CDF31D1-357D-447B-896F-0E94B310427D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{3D14CB9B-E28B-47AA-B0AB-3B4F47C5DE80}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" activeTab="1" xr2:uid="{E25BBD6F-6A55-41A2-8CA6-AC41BF09CE88}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{E25BBD6F-6A55-41A2-8CA6-AC41BF09CE88}"/>
   </bookViews>
   <sheets>
     <sheet name="Finance fucntions" sheetId="1" r:id="rId1"/>
@@ -232,7 +232,7 @@
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
   <numFmts count="2">
     <numFmt numFmtId="8" formatCode="&quot;₹&quot;\ #,##0.00;[Red]&quot;₹&quot;\ \-#,##0.00"/>
-    <numFmt numFmtId="165" formatCode="[$-F800]dddd\,\ mmmm\ dd\,\ yyyy"/>
+    <numFmt numFmtId="164" formatCode="[$-F800]dddd\,\ mmmm\ dd\,\ yyyy"/>
   </numFmts>
   <fonts count="1" x14ac:knownFonts="1">
     <font>
@@ -271,13 +271,13 @@
   </cellStyleXfs>
   <cellXfs count="6">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
+    <xf numFmtId="9" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
+    <xf numFmtId="8" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFill="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="9" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
-    <xf numFmtId="8" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
-    <xf numFmtId="165" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
-    <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFill="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -627,29 +627,29 @@
       <c r="D1" t="s">
         <v>0</v>
       </c>
-      <c r="E1" s="1" t="s">
+      <c r="E1" s="5" t="s">
         <v>8</v>
       </c>
-      <c r="F1" s="1"/>
-      <c r="G1" s="1"/>
-      <c r="H1" s="1"/>
-      <c r="I1" s="1"/>
-      <c r="J1" s="1"/>
-      <c r="K1" s="1"/>
-      <c r="L1" s="1"/>
-      <c r="M1" s="1"/>
+      <c r="F1" s="5"/>
+      <c r="G1" s="5"/>
+      <c r="H1" s="5"/>
+      <c r="I1" s="5"/>
+      <c r="J1" s="5"/>
+      <c r="K1" s="5"/>
+      <c r="L1" s="5"/>
+      <c r="M1" s="5"/>
     </row>
     <row r="2" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A2" t="s">
         <v>1</v>
       </c>
-      <c r="F2" s="1" t="s">
+      <c r="F2" s="5" t="s">
         <v>9</v>
       </c>
-      <c r="G2" s="1"/>
-      <c r="H2" s="1"/>
-      <c r="I2" s="1"/>
-      <c r="J2" s="1"/>
+      <c r="G2" s="5"/>
+      <c r="H2" s="5"/>
+      <c r="I2" s="5"/>
+      <c r="J2" s="5"/>
     </row>
     <row r="3" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A3" t="s">
@@ -695,7 +695,7 @@
       <c r="E8" t="s">
         <v>13</v>
       </c>
-      <c r="F8" s="2">
+      <c r="F8" s="1">
         <v>0.12</v>
       </c>
     </row>
@@ -711,7 +711,7 @@
       <c r="E10" t="s">
         <v>16</v>
       </c>
-      <c r="F10" s="3">
+      <c r="F10" s="2">
         <f>-PMT(12%/12,5*12,500000)</f>
         <v>11122.223842450885</v>
       </c>
@@ -736,7 +736,7 @@
       <c r="E17" t="s">
         <v>13</v>
       </c>
-      <c r="F17" s="2">
+      <c r="F17" s="1">
         <v>0.12</v>
       </c>
     </row>
@@ -752,7 +752,7 @@
       <c r="E19" t="s">
         <v>20</v>
       </c>
-      <c r="F19" s="3">
+      <c r="F19" s="2">
         <f>-IPMT(12%/12,34,5*12,500000)</f>
         <v>2620.3522923516161</v>
       </c>
@@ -777,10 +777,10 @@
       <c r="E27" t="s">
         <v>22</v>
       </c>
-      <c r="F27" s="2">
+      <c r="F27" s="1">
         <v>0.12</v>
       </c>
-      <c r="I27" s="3">
+      <c r="I27" s="2">
         <f>F29+F19</f>
         <v>11122.223842450885</v>
       </c>
@@ -797,7 +797,7 @@
       <c r="E29" t="s">
         <v>25</v>
       </c>
-      <c r="F29" s="3">
+      <c r="F29" s="2">
         <f>-PPMT(12%/12,34,5*12,500000)</f>
         <v>8501.8715500992694</v>
       </c>
@@ -811,7 +811,7 @@
       </c>
     </row>
     <row r="34" spans="4:6" x14ac:dyDescent="0.3">
-      <c r="E34" s="4">
+      <c r="E34" s="3">
         <f>EDATE("15-Feb-2026",-6)</f>
         <v>45884</v>
       </c>
@@ -859,7 +859,7 @@
       <c r="E43" t="s">
         <v>32</v>
       </c>
-      <c r="F43" s="2">
+      <c r="F43" s="1">
         <v>0.08</v>
       </c>
     </row>
@@ -872,13 +872,13 @@
       </c>
     </row>
     <row r="46" spans="4:6" x14ac:dyDescent="0.3">
-      <c r="E46" s="3">
+      <c r="E46" s="2">
         <f>FV(8%/12,10*12,-5000)</f>
         <v>914730.17590853572</v>
       </c>
     </row>
     <row r="47" spans="4:6" x14ac:dyDescent="0.3">
-      <c r="E47" s="3">
+      <c r="E47" s="2">
         <f>FV(8%/12,10*12,-5000,250000)</f>
         <v>359820.11727235711</v>
       </c>
@@ -892,7 +892,7 @@
       </c>
     </row>
     <row r="51" spans="4:6" x14ac:dyDescent="0.3">
-      <c r="E51" s="3">
+      <c r="E51" s="2">
         <f>PV(8%/12,10*12,-5000)</f>
         <v>412107.40446690557</v>
       </c>
@@ -930,7 +930,7 @@
       </c>
     </row>
     <row r="60" spans="4:6" x14ac:dyDescent="0.3">
-      <c r="F60" s="2">
+      <c r="F60" s="1">
         <f>RATE(5*12,-11122.22,500000)</f>
         <v>9.9999873269945166E-3</v>
       </c>
@@ -978,7 +978,7 @@
       <c r="E69" t="s">
         <v>32</v>
       </c>
-      <c r="F69" s="2">
+      <c r="F69" s="1">
         <v>0.12</v>
       </c>
     </row>
@@ -1015,16 +1015,16 @@
       <c r="E1">
         <v>34</v>
       </c>
-      <c r="I1" s="1" t="s">
+      <c r="I1" s="5" t="s">
         <v>50</v>
       </c>
-      <c r="J1" s="1"/>
-      <c r="K1" s="1"/>
-      <c r="M1" s="1" t="s">
+      <c r="J1" s="5"/>
+      <c r="K1" s="5"/>
+      <c r="M1" s="5" t="s">
         <v>54</v>
       </c>
-      <c r="N1" s="1"/>
-      <c r="O1" s="1"/>
+      <c r="N1" s="5"/>
+      <c r="O1" s="5"/>
     </row>
     <row r="2" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A2" t="s">
@@ -1034,22 +1034,22 @@
         <f>IF(E1&gt;=18,"Can vote","Can't vote")</f>
         <v>Can vote</v>
       </c>
-      <c r="I2" s="5" t="s">
+      <c r="I2" s="4" t="s">
         <v>51</v>
       </c>
-      <c r="J2" s="5" t="s">
+      <c r="J2" s="4" t="s">
         <v>52</v>
       </c>
-      <c r="K2" s="5" t="s">
+      <c r="K2" s="4" t="s">
         <v>53</v>
       </c>
-      <c r="M2" s="5" t="s">
+      <c r="M2" s="4" t="s">
         <v>51</v>
       </c>
-      <c r="N2" s="5" t="s">
+      <c r="N2" s="4" t="s">
         <v>52</v>
       </c>
-      <c r="O2" s="5" t="s">
+      <c r="O2" s="4" t="s">
         <v>53</v>
       </c>
     </row>

</xml_diff>